<commit_message>
access TO attributes from session; closes #1226
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97EDF513-64A8-4FFD-B4E9-A44E3D5ED978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2B296E-F107-4E50-A5B1-86019F5F3656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="23025" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -220,15 +220,6 @@
     <t>${session.timeKeeper}</t>
   </si>
   <si>
-    <t>${session.referee1}</t>
-  </si>
-  <si>
-    <t>${session.referee2}</t>
-  </si>
-  <si>
-    <t>${session.referee3}</t>
-  </si>
-  <si>
     <t>${session.announcer}</t>
   </si>
   <si>
@@ -425,6 +416,15 @@
   </si>
   <si>
     <t>${l.bestLifterScore}</t>
+  </si>
+  <si>
+    <t>${session.referee1AsTO} ${session.referee1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee2AsTO} ${session.referee2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee3AsTO} ${session.referee3AsTO.federationId}</t>
   </si>
 </sst>
 </file>
@@ -1314,13 +1314,36 @@
     <xf numFmtId="0" fontId="31" fillId="13" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1338,49 +1361,26 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="12" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1899,22 +1899,22 @@
       <c r="F1" s="49"/>
       <c r="G1" s="15"/>
       <c r="J1" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="102" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="102"/>
-      <c r="M1" s="102"/>
-      <c r="N1" s="102"/>
-      <c r="O1" s="102"/>
-      <c r="P1" s="102"/>
-      <c r="Q1" s="102"/>
-      <c r="R1" s="102"/>
-      <c r="S1" s="102"/>
-      <c r="T1" s="102"/>
-      <c r="U1" s="102"/>
-      <c r="V1" s="102"/>
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="109"/>
+      <c r="P1" s="109"/>
+      <c r="Q1" s="109"/>
+      <c r="R1" s="109"/>
+      <c r="S1" s="109"/>
+      <c r="T1" s="109"/>
+      <c r="U1" s="109"/>
+      <c r="V1" s="109"/>
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="53" t="s">
@@ -1923,10 +1923,10 @@
       <c r="B2" s="54"/>
       <c r="C2" s="4"/>
       <c r="J2" s="32" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="K2" s="55" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="L2" s="99"/>
       <c r="M2" s="56"/>
@@ -1935,7 +1935,7 @@
       <c r="P2" s="57"/>
       <c r="Q2" s="58"/>
       <c r="R2" s="32" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="S2" t="s">
         <v>18</v>
@@ -1949,19 +1949,19 @@
       </c>
       <c r="B3" s="60"/>
       <c r="J3" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" s="116" t="s">
-        <v>62</v>
-      </c>
-      <c r="L3" s="116"/>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
+        <v>31</v>
+      </c>
+      <c r="K3" s="106" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="106"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="61"/>
       <c r="R3" s="32" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="S3" s="62" t="s">
         <v>19</v>
@@ -1972,17 +1972,17 @@
     </row>
     <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="59" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B4" s="59"/>
       <c r="C4" s="48"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="J4" s="32" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="K4" s="100" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L4"/>
       <c r="M4" s="3"/>
@@ -1999,62 +1999,62 @@
       <c r="H6" s="7"/>
       <c r="I6" s="9"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="109" t="s">
-        <v>43</v>
-      </c>
-      <c r="L6" s="110"/>
-      <c r="M6" s="111"/>
+      <c r="K6" s="102" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6" s="115"/>
+      <c r="M6" s="103"/>
       <c r="N6" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="O6" s="102" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="115"/>
+      <c r="Q6" s="103"/>
+      <c r="R6" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="S6" s="112" t="s">
+        <v>47</v>
+      </c>
+      <c r="T6" s="110" t="s">
         <v>48</v>
       </c>
-      <c r="O6" s="109" t="s">
-        <v>44</v>
-      </c>
-      <c r="P6" s="110"/>
-      <c r="Q6" s="111"/>
-      <c r="R6" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="S6" s="106" t="s">
-        <v>50</v>
-      </c>
-      <c r="T6" s="104" t="s">
-        <v>51</v>
-      </c>
-      <c r="U6" s="118" t="s">
-        <v>91</v>
-      </c>
-      <c r="V6" s="119"/>
+      <c r="U6" s="116" t="s">
+        <v>88</v>
+      </c>
+      <c r="V6" s="117"/>
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="102" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="103"/>
+      <c r="G7" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="109" t="s">
+      <c r="I7" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="111"/>
-      <c r="G7" s="11" t="s">
+      <c r="J7" s="10" t="s">
         <v>39</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>42</v>
       </c>
       <c r="K7" s="10">
         <v>1</v>
@@ -2066,7 +2066,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="43" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="O7" s="10">
         <v>1</v>
@@ -2078,12 +2078,12 @@
         <v>3</v>
       </c>
       <c r="R7" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="S7" s="107"/>
-      <c r="T7" s="105"/>
-      <c r="U7" s="120"/>
-      <c r="V7" s="121"/>
+        <v>57</v>
+      </c>
+      <c r="S7" s="113"/>
+      <c r="T7" s="111"/>
+      <c r="U7" s="118"/>
+      <c r="V7" s="119"/>
     </row>
     <row r="8" spans="1:24" s="28" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="68"/>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="71" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B9" s="72"/>
       <c r="C9" s="73"/>
@@ -2130,7 +2130,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>1</v>
@@ -2138,10 +2138,10 @@
       <c r="D10" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="114" t="s">
+      <c r="E10" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="115"/>
+      <c r="F10" s="105"/>
       <c r="G10" s="66" t="s">
         <v>5</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="65" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="K10" s="27" t="s">
         <v>10</v>
@@ -2182,12 +2182,12 @@
         <v>7</v>
       </c>
       <c r="T10" s="46" t="s">
-        <v>88</v>
-      </c>
-      <c r="U10" s="112" t="s">
-        <v>92</v>
-      </c>
-      <c r="V10" s="113"/>
+        <v>85</v>
+      </c>
+      <c r="U10" s="120" t="s">
+        <v>89</v>
+      </c>
+      <c r="V10" s="121"/>
     </row>
     <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
@@ -2209,7 +2209,7 @@
     </row>
     <row r="12" spans="1:24" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="49" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="J12" s="50"/>
     </row>
@@ -2239,94 +2239,94 @@
     </row>
     <row r="14" spans="1:24" s="93" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B14" s="85"/>
       <c r="C14" s="86"/>
       <c r="D14" s="87" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E14" s="88" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F14" s="87" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H14" s="90"/>
       <c r="I14" s="87" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J14" s="84" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="K14" s="91"/>
       <c r="L14" s="85"/>
       <c r="M14" s="86"/>
       <c r="N14" s="84" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="O14" s="85"/>
       <c r="P14" s="92"/>
       <c r="Q14" s="84" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="R14" s="85"/>
       <c r="S14" s="84" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="T14" s="91"/>
       <c r="U14" s="84" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V14" s="92"/>
       <c r="X14" s="86"/>
     </row>
     <row r="15" spans="1:24" s="74" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="76" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B15" s="77"/>
       <c r="C15" s="78"/>
       <c r="D15" s="79" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E15" s="80" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F15" s="95" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="80" t="s">
         <v>83</v>
-      </c>
-      <c r="G15" s="80" t="s">
-        <v>86</v>
       </c>
       <c r="H15" s="78"/>
       <c r="I15" s="94" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J15" s="80" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="K15" s="77"/>
       <c r="L15" s="77"/>
       <c r="M15" s="78"/>
       <c r="N15" s="80" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="O15" s="77"/>
       <c r="P15" s="78"/>
       <c r="Q15" s="76" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="R15" s="77"/>
       <c r="S15" s="83" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T15" s="77"/>
       <c r="U15" s="82" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="V15" s="78"/>
       <c r="X15" s="78"/>
@@ -2335,23 +2335,23 @@
       <c r="A16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="117" t="s">
-        <v>53</v>
+      <c r="E16" s="107" t="s">
+        <v>50</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="15"/>
       <c r="I16" s="14"/>
-      <c r="J16" s="103" t="s">
-        <v>54</v>
-      </c>
-      <c r="K16" s="103"/>
+      <c r="J16" s="108" t="s">
+        <v>51</v>
+      </c>
+      <c r="K16" s="108"/>
       <c r="L16" s="14"/>
       <c r="N16" s="16"/>
       <c r="P16" s="14"/>
-      <c r="Q16" s="108" t="s">
-        <v>55</v>
-      </c>
-      <c r="R16" s="108"/>
+      <c r="Q16" s="114" t="s">
+        <v>52</v>
+      </c>
+      <c r="R16" s="114"/>
       <c r="S16" s="47"/>
       <c r="T16" s="14"/>
       <c r="U16" s="12"/>
@@ -2364,21 +2364,21 @@
     <row r="17" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="35" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D17" s="17"/>
-      <c r="E17" s="117"/>
+      <c r="E17" s="107"/>
       <c r="F17" s="41" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
-      <c r="J17" s="103"/>
-      <c r="K17" s="103"/>
+      <c r="J17" s="108"/>
+      <c r="K17" s="108"/>
       <c r="L17" s="41" t="s">
         <v>23</v>
       </c>
@@ -2386,10 +2386,10 @@
       <c r="N17" s="17"/>
       <c r="O17" s="17"/>
       <c r="P17" s="19"/>
-      <c r="Q17" s="108"/>
-      <c r="R17" s="108"/>
+      <c r="Q17" s="114"/>
+      <c r="R17" s="114"/>
       <c r="S17" s="41" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="T17" s="19"/>
       <c r="U17" s="17"/>
@@ -2425,10 +2425,10 @@
       <c r="E19" s="30"/>
       <c r="F19" s="14"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="103" t="s">
-        <v>58</v>
-      </c>
-      <c r="K19" s="103"/>
+      <c r="J19" s="108" t="s">
+        <v>55</v>
+      </c>
+      <c r="K19" s="108"/>
       <c r="M19"/>
       <c r="N19" s="1"/>
       <c r="O19" s="12"/>
@@ -2441,25 +2441,25 @@
     <row r="20" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="35" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="35" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="103"/>
-      <c r="K20" s="103"/>
+      <c r="J20" s="108"/>
+      <c r="K20" s="108"/>
       <c r="L20" s="41" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="M20" s="19"/>
       <c r="N20" s="17"/>
@@ -2510,17 +2510,17 @@
     <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="35" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D23" s="17"/>
       <c r="E23" s="35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G23" s="17"/>
       <c r="H23" s="17"/>
@@ -2880,11 +2880,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="J16:K17"/>
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="J19:K20"/>
     <mergeCell ref="T6:T7"/>
@@ -2894,6 +2889,11 @@
     <mergeCell ref="O6:Q6"/>
     <mergeCell ref="U6:V7"/>
     <mergeCell ref="U10:V10"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="J16:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:D8">
     <cfRule type="expression" dxfId="2" priority="7" stopIfTrue="1">
@@ -2911,7 +2911,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation showErrorMessage="1" sqref="F23 F20 C20 C17 S17 L17 F17 L20 C23 K4" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation showErrorMessage="1" sqref="F23 K4 C20 C17 S17 L17 F17 F20 C23 L20" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="G16 H11:H13" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
fixed the default templates to show the federaton id
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2B296E-F107-4E50-A5B1-86019F5F3656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F45054-5BCB-458D-B4F6-BDFF08953AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -217,12 +217,6 @@
     <t>${competition.federationWebSite}</t>
   </si>
   <si>
-    <t>${session.timeKeeper}</t>
-  </si>
-  <si>
-    <t>${session.announcer}</t>
-  </si>
-  <si>
     <t>${competition.competitionSite}</t>
   </si>
   <si>
@@ -367,18 +361,9 @@
     <t>${t.get("Results.RecordDate")}</t>
   </si>
   <si>
-    <t>${session.marshall} ${session.marshal2}</t>
-  </si>
-  <si>
     <t>${t.get("JuryPresident")}</t>
   </si>
   <si>
-    <t>${session.jury2} ${session.jury3} ${session.jury4} ${session.jury5}</t>
-  </si>
-  <si>
-    <t>${session.jury1}</t>
-  </si>
-  <si>
     <t>${t.get("Results.RecordAgeGroup")}</t>
   </si>
   <si>
@@ -400,9 +385,6 @@
     <t>${r.resRecordLift}</t>
   </si>
   <si>
-    <t>${session.technicalController} ${session.technicalController2}</t>
-  </si>
-  <si>
     <t>${l.totalRank &lt; 0 ? "inv." : (l.totalRank &gt; 0 ? l.totalRank : "" )}</t>
   </si>
   <si>
@@ -425,6 +407,24 @@
   </si>
   <si>
     <t>${session.referee3AsTO} ${session.referee3AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.announcerAsTO} ${session.referee1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.marshallAsTO} ${session.marshallAsTO.federationId} ${session.marshal2AsTO} ${session.marshal2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.timeKeeperAsTO} ${session.timeKeeperAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO} ${session.technicalControllerAsTO.federationId} ${session.technicalController2AsTO} ${session.technicalController2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.jury1AsTO} ${session.jury1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId}</t>
   </si>
 </sst>
 </file>
@@ -1314,14 +1314,60 @@
     <xf numFmtId="0" fontId="31" fillId="13" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -1336,52 +1382,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1899,22 +1899,22 @@
       <c r="F1" s="49"/>
       <c r="G1" s="15"/>
       <c r="J1" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="109"/>
-      <c r="M1" s="109"/>
-      <c r="N1" s="109"/>
-      <c r="O1" s="109"/>
-      <c r="P1" s="109"/>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="109"/>
-      <c r="S1" s="109"/>
-      <c r="T1" s="109"/>
-      <c r="U1" s="109"/>
-      <c r="V1" s="109"/>
+      <c r="L1" s="102"/>
+      <c r="M1" s="102"/>
+      <c r="N1" s="102"/>
+      <c r="O1" s="102"/>
+      <c r="P1" s="102"/>
+      <c r="Q1" s="102"/>
+      <c r="R1" s="102"/>
+      <c r="S1" s="102"/>
+      <c r="T1" s="102"/>
+      <c r="U1" s="102"/>
+      <c r="V1" s="102"/>
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="53" t="s">
@@ -1923,10 +1923,10 @@
       <c r="B2" s="54"/>
       <c r="C2" s="4"/>
       <c r="J2" s="32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K2" s="55" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L2" s="99"/>
       <c r="M2" s="56"/>
@@ -1935,7 +1935,7 @@
       <c r="P2" s="57"/>
       <c r="Q2" s="58"/>
       <c r="R2" s="32" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="S2" t="s">
         <v>18</v>
@@ -1949,19 +1949,19 @@
       </c>
       <c r="B3" s="60"/>
       <c r="J3" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="106" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" s="106"/>
-      <c r="M3" s="106"/>
-      <c r="N3" s="106"/>
-      <c r="O3" s="106"/>
+        <v>29</v>
+      </c>
+      <c r="K3" s="120" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" s="120"/>
+      <c r="M3" s="120"/>
+      <c r="N3" s="120"/>
+      <c r="O3" s="120"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="61"/>
       <c r="R3" s="32" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="S3" s="62" t="s">
         <v>19</v>
@@ -1972,17 +1972,17 @@
     </row>
     <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="59" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" s="59"/>
       <c r="C4" s="48"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="J4" s="32" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K4" s="100" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="L4"/>
       <c r="M4" s="3"/>
@@ -1999,62 +1999,62 @@
       <c r="H6" s="7"/>
       <c r="I6" s="9"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="102" t="s">
-        <v>40</v>
-      </c>
-      <c r="L6" s="115"/>
-      <c r="M6" s="103"/>
+      <c r="K6" s="109" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="110"/>
+      <c r="M6" s="111"/>
       <c r="N6" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="O6" s="109" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="110"/>
+      <c r="Q6" s="111"/>
+      <c r="R6" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="106" t="s">
         <v>45</v>
       </c>
-      <c r="O6" s="102" t="s">
-        <v>41</v>
-      </c>
-      <c r="P6" s="115"/>
-      <c r="Q6" s="103"/>
-      <c r="R6" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="S6" s="112" t="s">
-        <v>47</v>
-      </c>
-      <c r="T6" s="110" t="s">
-        <v>48</v>
-      </c>
-      <c r="U6" s="116" t="s">
-        <v>88</v>
-      </c>
-      <c r="V6" s="117"/>
+      <c r="T6" s="104" t="s">
+        <v>46</v>
+      </c>
+      <c r="U6" s="112" t="s">
+        <v>82</v>
+      </c>
+      <c r="V6" s="113"/>
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>44</v>
-      </c>
       <c r="D7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="109" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="111"/>
+      <c r="G7" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="H7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="103"/>
-      <c r="G7" s="11" t="s">
+      <c r="I7" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="J7" s="10" t="s">
         <v>37</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="K7" s="10">
         <v>1</v>
@@ -2066,7 +2066,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="43" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O7" s="10">
         <v>1</v>
@@ -2078,12 +2078,12 @@
         <v>3</v>
       </c>
       <c r="R7" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="S7" s="113"/>
-      <c r="T7" s="111"/>
-      <c r="U7" s="118"/>
-      <c r="V7" s="119"/>
+        <v>55</v>
+      </c>
+      <c r="S7" s="107"/>
+      <c r="T7" s="105"/>
+      <c r="U7" s="114"/>
+      <c r="V7" s="115"/>
     </row>
     <row r="8" spans="1:24" s="28" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="68"/>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="71" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B9" s="72"/>
       <c r="C9" s="73"/>
@@ -2130,7 +2130,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>1</v>
@@ -2138,10 +2138,10 @@
       <c r="D10" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="104" t="s">
+      <c r="E10" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="105"/>
+      <c r="F10" s="119"/>
       <c r="G10" s="66" t="s">
         <v>5</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="65" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K10" s="27" t="s">
         <v>10</v>
@@ -2182,12 +2182,12 @@
         <v>7</v>
       </c>
       <c r="T10" s="46" t="s">
-        <v>85</v>
-      </c>
-      <c r="U10" s="120" t="s">
-        <v>89</v>
-      </c>
-      <c r="V10" s="121"/>
+        <v>79</v>
+      </c>
+      <c r="U10" s="116" t="s">
+        <v>83</v>
+      </c>
+      <c r="V10" s="117"/>
     </row>
     <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
@@ -2209,7 +2209,7 @@
     </row>
     <row r="12" spans="1:24" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="49" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J12" s="50"/>
     </row>
@@ -2239,94 +2239,94 @@
     </row>
     <row r="14" spans="1:24" s="93" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B14" s="85"/>
       <c r="C14" s="86"/>
       <c r="D14" s="87" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E14" s="88" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F14" s="87" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="H14" s="90"/>
       <c r="I14" s="87" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J14" s="84" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K14" s="91"/>
       <c r="L14" s="85"/>
       <c r="M14" s="86"/>
       <c r="N14" s="84" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="O14" s="85"/>
       <c r="P14" s="92"/>
       <c r="Q14" s="84" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="R14" s="85"/>
       <c r="S14" s="84" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T14" s="91"/>
       <c r="U14" s="84" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="V14" s="92"/>
       <c r="X14" s="86"/>
     </row>
     <row r="15" spans="1:24" s="74" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="76" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B15" s="77"/>
       <c r="C15" s="78"/>
       <c r="D15" s="79" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E15" s="80" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F15" s="95" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G15" s="80" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H15" s="78"/>
       <c r="I15" s="94" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J15" s="80" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="K15" s="77"/>
       <c r="L15" s="77"/>
       <c r="M15" s="78"/>
       <c r="N15" s="80" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O15" s="77"/>
       <c r="P15" s="78"/>
       <c r="Q15" s="76" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="R15" s="77"/>
       <c r="S15" s="83" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T15" s="77"/>
       <c r="U15" s="82" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="V15" s="78"/>
       <c r="X15" s="78"/>
@@ -2335,23 +2335,23 @@
       <c r="A16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="107" t="s">
-        <v>50</v>
+      <c r="E16" s="121" t="s">
+        <v>48</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="15"/>
       <c r="I16" s="14"/>
-      <c r="J16" s="108" t="s">
-        <v>51</v>
-      </c>
-      <c r="K16" s="108"/>
+      <c r="J16" s="103" t="s">
+        <v>49</v>
+      </c>
+      <c r="K16" s="103"/>
       <c r="L16" s="14"/>
       <c r="N16" s="16"/>
       <c r="P16" s="14"/>
-      <c r="Q16" s="114" t="s">
-        <v>52</v>
-      </c>
-      <c r="R16" s="114"/>
+      <c r="Q16" s="108" t="s">
+        <v>50</v>
+      </c>
+      <c r="R16" s="108"/>
       <c r="S16" s="47"/>
       <c r="T16" s="14"/>
       <c r="U16" s="12"/>
@@ -2364,32 +2364,32 @@
     <row r="17" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="35" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="D17" s="17"/>
-      <c r="E17" s="107"/>
+      <c r="E17" s="121"/>
       <c r="F17" s="41" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
-      <c r="J17" s="108"/>
-      <c r="K17" s="108"/>
+      <c r="J17" s="103"/>
+      <c r="K17" s="103"/>
       <c r="L17" s="41" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
       <c r="O17" s="17"/>
       <c r="P17" s="19"/>
-      <c r="Q17" s="114"/>
-      <c r="R17" s="114"/>
+      <c r="Q17" s="108"/>
+      <c r="R17" s="108"/>
       <c r="S17" s="41" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="T17" s="19"/>
       <c r="U17" s="17"/>
@@ -2425,10 +2425,10 @@
       <c r="E19" s="30"/>
       <c r="F19" s="14"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="108" t="s">
-        <v>55</v>
-      </c>
-      <c r="K19" s="108"/>
+      <c r="J19" s="103" t="s">
+        <v>53</v>
+      </c>
+      <c r="K19" s="103"/>
       <c r="M19"/>
       <c r="N19" s="1"/>
       <c r="O19" s="12"/>
@@ -2441,25 +2441,25 @@
     <row r="20" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="35" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="35" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="108"/>
-      <c r="K20" s="108"/>
+      <c r="J20" s="103"/>
+      <c r="K20" s="103"/>
       <c r="L20" s="41" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="M20" s="19"/>
       <c r="N20" s="17"/>
@@ -2510,17 +2510,17 @@
     <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="35" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="D23" s="17"/>
       <c r="E23" s="35" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="G23" s="17"/>
       <c r="H23" s="17"/>
@@ -2880,6 +2880,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="J16:K17"/>
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="J19:K20"/>
     <mergeCell ref="T6:T7"/>
@@ -2889,11 +2894,6 @@
     <mergeCell ref="O6:Q6"/>
     <mergeCell ref="U6:V7"/>
     <mergeCell ref="U10:V10"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="J16:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:D8">
     <cfRule type="expression" dxfId="2" priority="7" stopIfTrue="1">

</xml_diff>

<commit_message>
fix for missing new records section
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\protocol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E79D63-87CE-490F-9594-BC9C3B2706AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3741C88B-9EB3-4005-8420-839323C22635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11805" yWindow="4170" windowWidth="25065" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -124,7 +124,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:if(condition="records != null" lastCell="V15")</t>
+          <t>jx:if(condition="group.records.size() &gt; 0"  lastCell="V15")</t>
         </r>
       </text>
     </comment>
@@ -137,7 +137,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:each(items="records" var="r" lastCell="V15")</t>
+          <t>jx:each(items="group.records" var="r" lastCell="V15")</t>
         </r>
       </text>
     </comment>
@@ -316,121 +316,121 @@
     <t>${t.get("Results.CJ_abbrev")}</t>
   </si>
   <si>
+    <t>${competition.localizedCompetitionDate}</t>
+  </si>
+  <si>
+    <t>${r.recordFederation}</t>
+  </si>
+  <si>
+    <t>${r.recordName}</t>
+  </si>
+  <si>
+    <t>${r.recordValue}</t>
+  </si>
+  <si>
+    <t>${r.nation}</t>
+  </si>
+  <si>
+    <t>${r.recordDateAsString}</t>
+  </si>
+  <si>
+    <t>${r.groupNameString}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ${r.birth}</t>
+  </si>
+  <si>
+    <t>${t.get("Preparation.Records")}</t>
+  </si>
+  <si>
+    <t>${t.get("Group")}</t>
+  </si>
+  <si>
+    <t>${t.get("Name")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordName")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordWeight")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordDate")}</t>
+  </si>
+  <si>
+    <t>${t.get("JuryPresident")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordAgeGroup")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordFederation")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordKind")}</t>
+  </si>
+  <si>
+    <t>${r.bwCatString}</t>
+  </si>
+  <si>
+    <t>${r.ageGrp} ${r.gender}</t>
+  </si>
+  <si>
+    <t>${r.resAthleteName}</t>
+  </si>
+  <si>
+    <t>${r.resRecordLift}</t>
+  </si>
+  <si>
+    <t>${l.totalRank &lt; 0 ? "inv." : (l.totalRank &gt; 0 ? l.totalRank : "" )}</t>
+  </si>
+  <si>
+    <t>${session != null ? t.get("Group") + " :" : ""}</t>
+  </si>
+  <si>
+    <t>${session.name}</t>
+  </si>
+  <si>
+    <t>${bestRankingTitle}</t>
+  </si>
+  <si>
+    <t>${l.bestLifterScore}</t>
+  </si>
+  <si>
+    <t>${session.referee1AsTO} ${session.referee1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee2AsTO} ${session.referee2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee3AsTO} ${session.referee3AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.marshallAsTO} ${session.marshallAsTO.federationId} ${session.marshal2AsTO} ${session.marshal2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.timeKeeperAsTO} ${session.timeKeeperAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO} ${session.technicalControllerAsTO.federationId} ${session.technicalController2AsTO} ${session.technicalController2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.jury1AsTO} ${session.jury1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.announcerAsTO} ${session.announcerAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("Reserve")}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO} ${session.reserveAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId} ${session.reserveJuryAsTO != null ? "("+t.get("Reserve")+") "+session.reserveJuryAsTO+" "+session.reserveJuryAsTO.federationId : ""}</t>
+  </si>
+  <si>
     <t>${group.item.category}</t>
-  </si>
-  <si>
-    <t>${competition.localizedCompetitionDate}</t>
-  </si>
-  <si>
-    <t>${r.recordFederation}</t>
-  </si>
-  <si>
-    <t>${r.recordName}</t>
-  </si>
-  <si>
-    <t>${r.recordValue}</t>
-  </si>
-  <si>
-    <t>${r.nation}</t>
-  </si>
-  <si>
-    <t>${r.recordDateAsString}</t>
-  </si>
-  <si>
-    <t>${r.groupNameString}</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ${r.birth}</t>
-  </si>
-  <si>
-    <t>${t.get("Preparation.Records")}</t>
-  </si>
-  <si>
-    <t>${t.get("Group")}</t>
-  </si>
-  <si>
-    <t>${t.get("Name")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordName")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordWeight")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordDate")}</t>
-  </si>
-  <si>
-    <t>${t.get("JuryPresident")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordAgeGroup")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordFederation")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.RecordKind")}</t>
-  </si>
-  <si>
-    <t>${r.bwCatString}</t>
-  </si>
-  <si>
-    <t>${r.ageGrp} ${r.gender}</t>
-  </si>
-  <si>
-    <t>${r.resAthleteName}</t>
-  </si>
-  <si>
-    <t>${r.resRecordLift}</t>
-  </si>
-  <si>
-    <t>${l.totalRank &lt; 0 ? "inv." : (l.totalRank &gt; 0 ? l.totalRank : "" )}</t>
-  </si>
-  <si>
-    <t>${session != null ? t.get("Group") + " :" : ""}</t>
-  </si>
-  <si>
-    <t>${session.name}</t>
-  </si>
-  <si>
-    <t>${bestRankingTitle}</t>
-  </si>
-  <si>
-    <t>${l.bestLifterScore}</t>
-  </si>
-  <si>
-    <t>${session.referee1AsTO} ${session.referee1AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.referee2AsTO} ${session.referee2AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.referee3AsTO} ${session.referee3AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.marshallAsTO} ${session.marshallAsTO.federationId} ${session.marshal2AsTO} ${session.marshal2AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.timeKeeperAsTO} ${session.timeKeeperAsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.technicalControllerAsTO} ${session.technicalControllerAsTO.federationId} ${session.technicalController2AsTO} ${session.technicalController2AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.jury1AsTO} ${session.jury1AsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.announcerAsTO} ${session.announcerAsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${t.get("Reserve")}</t>
-  </si>
-  <si>
-    <t>${session.reserveAsTO} ${session.reserveAsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId} ${session.reserveJuryAsTO != null ? "("+t.get("Reserve")+") "+session.reserveJuryAsTO+" "+session.reserveJuryAsTO.federationId : ""}</t>
   </si>
 </sst>
 </file>
@@ -1963,7 +1963,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="123" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L3" s="123"/>
       <c r="M3" s="123"/>
@@ -1990,10 +1990,10 @@
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="J4" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4" s="100" t="s">
         <v>80</v>
-      </c>
-      <c r="K4" s="100" t="s">
-        <v>81</v>
       </c>
       <c r="L4"/>
       <c r="M4" s="3"/>
@@ -2033,7 +2033,7 @@
         <v>46</v>
       </c>
       <c r="U6" s="115" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V6" s="116"/>
       <c r="X6"/>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="71" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="B9" s="72"/>
       <c r="C9" s="73"/>
@@ -2193,10 +2193,10 @@
         <v>7</v>
       </c>
       <c r="T10" s="46" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U10" s="119" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="V10" s="120"/>
     </row>
@@ -2220,7 +2220,7 @@
     </row>
     <row r="12" spans="1:24" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="49" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J12" s="50"/>
     </row>
@@ -2250,28 +2250,28 @@
     </row>
     <row r="14" spans="1:24" s="93" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="85"/>
       <c r="C14" s="86"/>
       <c r="D14" s="87" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14" s="88" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F14" s="87" t="s">
         <v>34</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H14" s="90"/>
       <c r="I14" s="87" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J14" s="84" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="91"/>
       <c r="L14" s="85"/>
@@ -2286,58 +2286,58 @@
       </c>
       <c r="R14" s="85"/>
       <c r="S14" s="84" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T14" s="91"/>
       <c r="U14" s="84" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="V14" s="92"/>
       <c r="X14" s="86"/>
     </row>
     <row r="15" spans="1:24" s="74" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="76" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="77"/>
       <c r="C15" s="78"/>
       <c r="D15" s="79" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E15" s="80" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F15" s="95" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G15" s="80" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H15" s="78"/>
       <c r="I15" s="94" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J15" s="80" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K15" s="77"/>
       <c r="L15" s="77"/>
       <c r="M15" s="78"/>
       <c r="N15" s="80" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O15" s="77"/>
       <c r="P15" s="78"/>
       <c r="Q15" s="76" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="R15" s="77"/>
       <c r="S15" s="83" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="T15" s="77"/>
       <c r="U15" s="82" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V15" s="78"/>
       <c r="X15" s="78"/>
@@ -2378,12 +2378,12 @@
         <v>47</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D17" s="17"/>
       <c r="E17" s="124"/>
       <c r="F17" s="41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
@@ -2391,7 +2391,7 @@
       <c r="J17" s="106"/>
       <c r="K17" s="106"/>
       <c r="L17" s="41" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
@@ -2400,7 +2400,7 @@
       <c r="Q17" s="111"/>
       <c r="R17" s="111"/>
       <c r="S17" s="41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="T17" s="19"/>
       <c r="U17" s="17"/>
@@ -2442,7 +2442,7 @@
       <c r="N19" s="1"/>
       <c r="O19" s="12"/>
       <c r="Q19" s="106" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R19" s="106"/>
       <c r="S19" s="1"/>
@@ -2456,14 +2456,14 @@
         <v>51</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="35" t="s">
         <v>52</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
@@ -2471,7 +2471,7 @@
       <c r="J20" s="106"/>
       <c r="K20" s="106"/>
       <c r="L20" s="41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M20" s="19"/>
       <c r="N20" s="17"/>
@@ -2480,7 +2480,7 @@
       <c r="Q20" s="106"/>
       <c r="R20" s="106"/>
       <c r="S20" s="41" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="T20" s="19"/>
       <c r="U20" s="17"/>
@@ -2525,17 +2525,17 @@
     <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" s="17"/>
       <c r="E23" s="35" t="s">
         <v>54</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G23" s="17"/>
       <c r="H23" s="17"/>

</xml_diff>

<commit_message>
records on single-category results sheet; closes jxls1 iteration over category records Fixes #1382
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3741C88B-9EB3-4005-8420-839323C22635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5608072-C9DF-40CE-AEE1-967763E8FBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11805" yWindow="4170" windowWidth="25065" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="9690" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -721,7 +721,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -771,19 +771,6 @@
         <color indexed="8"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -912,19 +899,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color indexed="8"/>
@@ -1006,14 +980,29 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
       </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1026,7 +1015,7 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1052,7 +1041,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1119,23 +1108,9 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1158,34 +1133,20 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1226,24 +1187,14 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1251,62 +1202,62 @@
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="12" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="12" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="13" xfId="12" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="12" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="14" xfId="12" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="14" xfId="12" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="12" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="15" xfId="12" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1317,82 +1268,128 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1900,99 +1897,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
       <c r="G1" s="15"/>
-      <c r="J1" s="32" t="s">
+      <c r="J1" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="K1" s="105" t="s">
+      <c r="K1" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="105"/>
-      <c r="M1" s="105"/>
-      <c r="N1" s="105"/>
-      <c r="O1" s="105"/>
-      <c r="P1" s="105"/>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105"/>
-      <c r="T1" s="105"/>
-      <c r="U1" s="105"/>
-      <c r="V1" s="105"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="94"/>
+      <c r="R1" s="94"/>
+      <c r="S1" s="94"/>
+      <c r="T1" s="94"/>
+      <c r="U1" s="94"/>
+      <c r="V1" s="94"/>
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="46"/>
       <c r="C2" s="4"/>
-      <c r="J2" s="32" t="s">
+      <c r="J2" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="55" t="s">
+      <c r="K2" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="99"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="57"/>
-      <c r="Q2" s="58"/>
-      <c r="R2" s="32" t="s">
+      <c r="L2" s="88"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="50"/>
+      <c r="R2" s="28" t="s">
         <v>30</v>
       </c>
       <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="58"/>
-      <c r="U2" s="58"/>
+      <c r="T2" s="50"/>
+      <c r="U2" s="50"/>
     </row>
     <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="J3" s="32" t="s">
+      <c r="B3" s="52"/>
+      <c r="J3" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="123" t="s">
+      <c r="K3" s="108" t="s">
         <v>56</v>
       </c>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
+      <c r="L3" s="108"/>
+      <c r="M3" s="108"/>
+      <c r="N3" s="108"/>
+      <c r="O3" s="108"/>
       <c r="P3" s="6"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="32" t="s">
+      <c r="Q3" s="53"/>
+      <c r="R3" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="S3" s="62" t="s">
+      <c r="S3" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="T3" s="63"/>
-      <c r="U3" s="63"/>
-      <c r="V3" s="96"/>
+      <c r="T3" s="55"/>
+      <c r="U3" s="55"/>
+      <c r="V3" s="85"/>
     </row>
     <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="48"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="40"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
-      <c r="J4" s="32" t="s">
+      <c r="J4" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="100" t="s">
+      <c r="K4" s="89" t="s">
         <v>80</v>
       </c>
       <c r="L4"/>
@@ -2000,8 +1997,8 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="Q4"/>
-      <c r="R4" s="32"/>
-      <c r="S4" s="64"/>
+      <c r="R4" s="28"/>
+      <c r="S4" s="56"/>
     </row>
     <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2010,32 +2007,32 @@
       <c r="H6" s="7"/>
       <c r="I6" s="9"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="112" t="s">
+      <c r="K6" s="101" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="113"/>
-      <c r="M6" s="114"/>
-      <c r="N6" s="42" t="s">
+      <c r="L6" s="102"/>
+      <c r="M6" s="103"/>
+      <c r="N6" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="O6" s="112" t="s">
+      <c r="O6" s="101" t="s">
         <v>39</v>
       </c>
-      <c r="P6" s="113"/>
-      <c r="Q6" s="114"/>
-      <c r="R6" s="44" t="s">
+      <c r="P6" s="102"/>
+      <c r="Q6" s="103"/>
+      <c r="R6" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="S6" s="109" t="s">
+      <c r="S6" s="98" t="s">
         <v>45</v>
       </c>
-      <c r="T6" s="107" t="s">
+      <c r="T6" s="96" t="s">
         <v>46</v>
       </c>
-      <c r="U6" s="115" t="s">
+      <c r="U6" s="104" t="s">
         <v>81</v>
       </c>
-      <c r="V6" s="116"/>
+      <c r="V6" s="105"/>
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2051,10 +2048,10 @@
       <c r="D7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="112" t="s">
+      <c r="E7" s="101" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="114"/>
+      <c r="F7" s="103"/>
       <c r="G7" s="11" t="s">
         <v>34</v>
       </c>
@@ -2076,7 +2073,7 @@
       <c r="M7" s="10">
         <v>3</v>
       </c>
-      <c r="N7" s="43" t="s">
+      <c r="N7" s="36" t="s">
         <v>44</v>
       </c>
       <c r="O7" s="10">
@@ -2088,282 +2085,309 @@
       <c r="Q7" s="10">
         <v>3</v>
       </c>
-      <c r="R7" s="45" t="s">
+      <c r="R7" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="S7" s="110"/>
-      <c r="T7" s="108"/>
-      <c r="U7" s="117"/>
-      <c r="V7" s="118"/>
-    </row>
-    <row r="8" spans="1:24" s="28" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="68"/>
-      <c r="B8" s="68"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="69"/>
-      <c r="K8" s="70"/>
+      <c r="S7" s="99"/>
+      <c r="T7" s="97"/>
+      <c r="U7" s="106"/>
+      <c r="V7" s="107"/>
+    </row>
+    <row r="8" spans="1:24" s="25" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="57"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="58"/>
+      <c r="K8" s="59"/>
     </row>
     <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="71" t="s">
+      <c r="A9" s="60" t="s">
         <v>94</v>
       </c>
-      <c r="B9" s="72"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73"/>
-      <c r="F9" s="73"/>
-      <c r="G9" s="73"/>
-      <c r="H9" s="73"/>
-      <c r="I9" s="73"/>
-      <c r="J9" s="73"/>
-      <c r="K9" s="73"/>
-      <c r="L9" s="73"/>
-      <c r="M9" s="73"/>
-      <c r="N9" s="73"/>
-      <c r="O9" s="73"/>
-      <c r="P9" s="73"/>
-      <c r="Q9" s="73"/>
-      <c r="R9" s="73"/>
-      <c r="S9" s="73"/>
-      <c r="T9" s="73"/>
-      <c r="U9" s="73"/>
-      <c r="V9" s="101"/>
+      <c r="B9" s="61"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+      <c r="L9" s="62"/>
+      <c r="M9" s="62"/>
+      <c r="N9" s="62"/>
+      <c r="O9" s="62"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="62"/>
+      <c r="R9" s="62"/>
+      <c r="S9" s="62"/>
+      <c r="T9" s="62"/>
+      <c r="U9" s="62"/>
+      <c r="V9" s="90"/>
       <c r="X9"/>
     </row>
-    <row r="10" spans="1:24" s="28" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:24" s="25" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="117" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="121" t="s">
+      <c r="E10" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="122"/>
-      <c r="G10" s="66" t="s">
+      <c r="F10" s="113"/>
+      <c r="G10" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="38" t="s">
+      <c r="H10" s="119" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="67" t="s">
+      <c r="I10" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="65" t="s">
+      <c r="J10" s="121" t="s">
         <v>26</v>
       </c>
-      <c r="K10" s="27" t="s">
+      <c r="K10" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="L10" s="27" t="s">
+      <c r="L10" s="122" t="s">
         <v>11</v>
       </c>
-      <c r="M10" s="27" t="s">
+      <c r="M10" s="122" t="s">
         <v>12</v>
       </c>
-      <c r="N10" s="29" t="s">
+      <c r="N10" s="123" t="s">
         <v>8</v>
       </c>
-      <c r="O10" s="27" t="s">
+      <c r="O10" s="122" t="s">
         <v>13</v>
       </c>
-      <c r="P10" s="27" t="s">
+      <c r="P10" s="122" t="s">
         <v>14</v>
       </c>
-      <c r="Q10" s="27" t="s">
+      <c r="Q10" s="122" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="39" t="s">
+      <c r="R10" s="124" t="s">
         <v>9</v>
       </c>
-      <c r="S10" s="40" t="s">
+      <c r="S10" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="T10" s="46" t="s">
+      <c r="T10" s="126" t="s">
         <v>78</v>
       </c>
-      <c r="U10" s="119" t="s">
+      <c r="U10" s="127" t="s">
         <v>82</v>
       </c>
-      <c r="V10" s="120"/>
+      <c r="V10" s="128"/>
     </row>
     <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11"/>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11"/>
-      <c r="K11"/>
-      <c r="L11"/>
-      <c r="M11"/>
-      <c r="O11"/>
-      <c r="P11"/>
-      <c r="Q11"/>
-      <c r="R11"/>
-      <c r="T11"/>
-      <c r="U11"/>
-      <c r="V11"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="115"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="114"/>
+      <c r="M11" s="114"/>
+      <c r="N11" s="114"/>
+      <c r="O11" s="114"/>
+      <c r="P11" s="114"/>
+      <c r="Q11" s="114"/>
+      <c r="R11" s="114"/>
+      <c r="S11" s="114"/>
+      <c r="T11" s="114"/>
+      <c r="U11" s="114"/>
+      <c r="V11" s="114"/>
       <c r="W11"/>
       <c r="X11"/>
     </row>
-    <row r="12" spans="1:24" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="49" t="s">
+    <row r="12" spans="1:24" s="41" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="J12" s="50"/>
-    </row>
-    <row r="13" spans="1:24" s="49" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="75"/>
-      <c r="B13" s="75"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="75"/>
-      <c r="G13" s="75"/>
-      <c r="H13" s="75"/>
-      <c r="I13" s="75"/>
-      <c r="J13" s="81"/>
-      <c r="K13" s="75"/>
-      <c r="L13" s="75"/>
-      <c r="M13" s="75"/>
-      <c r="N13" s="75"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="81"/>
-      <c r="Q13" s="81"/>
-      <c r="R13" s="81"/>
-      <c r="S13" s="75"/>
-      <c r="T13" s="75"/>
-      <c r="U13" s="81"/>
-      <c r="V13" s="81"/>
-    </row>
-    <row r="14" spans="1:24" s="93" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A14" s="84" t="s">
+      <c r="B12" s="110"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="116"/>
+      <c r="K12" s="110"/>
+      <c r="L12" s="110"/>
+      <c r="M12" s="110"/>
+      <c r="N12" s="110"/>
+      <c r="O12" s="110"/>
+      <c r="P12" s="110"/>
+      <c r="Q12" s="110"/>
+      <c r="R12" s="110"/>
+      <c r="S12" s="110"/>
+      <c r="T12" s="110"/>
+      <c r="U12" s="110"/>
+      <c r="V12" s="110"/>
+    </row>
+    <row r="13" spans="1:24" s="41" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="64"/>
+      <c r="H13" s="64"/>
+      <c r="I13" s="64"/>
+      <c r="J13" s="70"/>
+      <c r="K13" s="64"/>
+      <c r="L13" s="64"/>
+      <c r="M13" s="64"/>
+      <c r="N13" s="64"/>
+      <c r="O13" s="64"/>
+      <c r="P13" s="70"/>
+      <c r="Q13" s="70"/>
+      <c r="R13" s="70"/>
+      <c r="S13" s="64"/>
+      <c r="T13" s="64"/>
+      <c r="U13" s="70"/>
+      <c r="V13" s="70"/>
+    </row>
+    <row r="14" spans="1:24" s="82" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A14" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="85"/>
-      <c r="C14" s="86"/>
-      <c r="D14" s="87" t="s">
+      <c r="B14" s="74"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="76" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="88" t="s">
+      <c r="E14" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="F14" s="87" t="s">
+      <c r="F14" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="G14" s="89" t="s">
+      <c r="G14" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="H14" s="90"/>
-      <c r="I14" s="87" t="s">
+      <c r="H14" s="79"/>
+      <c r="I14" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="J14" s="84" t="s">
+      <c r="J14" s="73" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="91"/>
-      <c r="L14" s="85"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="84" t="s">
+      <c r="K14" s="80"/>
+      <c r="L14" s="74"/>
+      <c r="M14" s="75"/>
+      <c r="N14" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="O14" s="85"/>
-      <c r="P14" s="92"/>
-      <c r="Q14" s="84" t="s">
+      <c r="O14" s="74"/>
+      <c r="P14" s="81"/>
+      <c r="Q14" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="85"/>
-      <c r="S14" s="84" t="s">
+      <c r="R14" s="74"/>
+      <c r="S14" s="73" t="s">
         <v>65</v>
       </c>
-      <c r="T14" s="91"/>
-      <c r="U14" s="84" t="s">
+      <c r="T14" s="80"/>
+      <c r="U14" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="V14" s="92"/>
-      <c r="X14" s="86"/>
-    </row>
-    <row r="15" spans="1:24" s="74" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="76" t="s">
+      <c r="V14" s="81"/>
+      <c r="X14" s="75"/>
+    </row>
+    <row r="15" spans="1:24" s="63" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="78"/>
-      <c r="D15" s="79" t="s">
+      <c r="B15" s="66"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="80" t="s">
+      <c r="E15" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="95" t="s">
+      <c r="F15" s="84" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="80" t="s">
+      <c r="G15" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="H15" s="78"/>
-      <c r="I15" s="94" t="s">
+      <c r="H15" s="67"/>
+      <c r="I15" s="83" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="80" t="s">
+      <c r="J15" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="K15" s="77"/>
-      <c r="L15" s="77"/>
-      <c r="M15" s="78"/>
-      <c r="N15" s="80" t="s">
+      <c r="K15" s="66"/>
+      <c r="L15" s="66"/>
+      <c r="M15" s="67"/>
+      <c r="N15" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="77"/>
-      <c r="P15" s="78"/>
-      <c r="Q15" s="76" t="s">
+      <c r="O15" s="66"/>
+      <c r="P15" s="67"/>
+      <c r="Q15" s="65" t="s">
         <v>63</v>
       </c>
-      <c r="R15" s="77"/>
-      <c r="S15" s="83" t="s">
+      <c r="R15" s="66"/>
+      <c r="S15" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="T15" s="77"/>
-      <c r="U15" s="82" t="s">
+      <c r="T15" s="66"/>
+      <c r="U15" s="71" t="s">
         <v>61</v>
       </c>
-      <c r="V15" s="78"/>
-      <c r="X15" s="78"/>
+      <c r="V15" s="67"/>
+      <c r="X15" s="67"/>
     </row>
     <row r="16" spans="1:24" s="13" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="124" t="s">
+      <c r="E16" s="109" t="s">
         <v>48</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="15"/>
       <c r="I16" s="14"/>
-      <c r="J16" s="106" t="s">
+      <c r="J16" s="95" t="s">
         <v>49</v>
       </c>
-      <c r="K16" s="106"/>
+      <c r="K16" s="95"/>
       <c r="L16" s="14"/>
       <c r="N16" s="16"/>
       <c r="P16" s="14"/>
-      <c r="Q16" s="111" t="s">
+      <c r="Q16" s="100" t="s">
         <v>50</v>
       </c>
-      <c r="R16" s="111"/>
-      <c r="S16" s="47"/>
+      <c r="R16" s="100"/>
+      <c r="S16" s="39"/>
       <c r="T16" s="14"/>
       <c r="U16" s="12"/>
       <c r="V16" s="16"/>
@@ -2374,77 +2398,77 @@
     </row>
     <row r="17" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C17" s="34" t="s">
         <v>90</v>
       </c>
       <c r="D17" s="17"/>
-      <c r="E17" s="124"/>
-      <c r="F17" s="41" t="s">
+      <c r="E17" s="109"/>
+      <c r="F17" s="34" t="s">
         <v>86</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
-      <c r="J17" s="106"/>
-      <c r="K17" s="106"/>
-      <c r="L17" s="41" t="s">
+      <c r="J17" s="95"/>
+      <c r="K17" s="95"/>
+      <c r="L17" s="34" t="s">
         <v>87</v>
       </c>
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
       <c r="O17" s="17"/>
       <c r="P17" s="19"/>
-      <c r="Q17" s="111"/>
-      <c r="R17" s="111"/>
-      <c r="S17" s="41" t="s">
+      <c r="Q17" s="100"/>
+      <c r="R17" s="100"/>
+      <c r="S17" s="34" t="s">
         <v>88</v>
       </c>
       <c r="T17" s="19"/>
       <c r="U17" s="17"/>
-      <c r="V17" s="51"/>
+      <c r="V17" s="43"/>
       <c r="W17"/>
     </row>
     <row r="18" spans="1:24" s="20" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="A18" s="21"/>
-      <c r="B18" s="33"/>
-      <c r="D18" s="37"/>
+      <c r="B18" s="29"/>
+      <c r="D18" s="33"/>
       <c r="E18" s="18"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="37"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
       <c r="I18" s="21"/>
       <c r="K18" s="18"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="33"/>
+      <c r="P18" s="33"/>
       <c r="Q18" s="21"/>
-      <c r="S18" s="37"/>
-      <c r="T18" s="37"/>
-      <c r="U18" s="37"/>
-      <c r="V18" s="98"/>
+      <c r="S18" s="33"/>
+      <c r="T18" s="33"/>
+      <c r="U18" s="33"/>
+      <c r="V18" s="87"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="31"/>
+      <c r="B19" s="27"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="30"/>
+      <c r="E19" s="26"/>
       <c r="F19" s="14"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="106" t="s">
+      <c r="J19" s="95" t="s">
         <v>53</v>
       </c>
-      <c r="K19" s="106"/>
+      <c r="K19" s="95"/>
       <c r="M19"/>
       <c r="N19" s="1"/>
       <c r="O19" s="12"/>
-      <c r="Q19" s="106" t="s">
+      <c r="Q19" s="95" t="s">
         <v>91</v>
       </c>
-      <c r="R19" s="106"/>
+      <c r="R19" s="95"/>
       <c r="S19" s="1"/>
       <c r="T19"/>
       <c r="V19" s="12"/>
@@ -2452,34 +2476,34 @@
     </row>
     <row r="20" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="35" t="s">
+      <c r="B20" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="34" t="s">
         <v>83</v>
       </c>
       <c r="D20" s="17"/>
-      <c r="E20" s="35" t="s">
+      <c r="E20" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="F20" s="41" t="s">
+      <c r="F20" s="34" t="s">
         <v>84</v>
       </c>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="106"/>
-      <c r="K20" s="106"/>
-      <c r="L20" s="41" t="s">
+      <c r="J20" s="95"/>
+      <c r="K20" s="95"/>
+      <c r="L20" s="34" t="s">
         <v>85</v>
       </c>
       <c r="M20" s="19"/>
       <c r="N20" s="17"/>
       <c r="O20" s="17"/>
       <c r="P20" s="17"/>
-      <c r="Q20" s="106"/>
-      <c r="R20" s="106"/>
-      <c r="S20" s="41" t="s">
+      <c r="Q20" s="95"/>
+      <c r="R20" s="95"/>
+      <c r="S20" s="34" t="s">
         <v>92</v>
       </c>
       <c r="T20" s="19"/>
@@ -2489,52 +2513,52 @@
     </row>
     <row r="21" spans="1:24" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
-      <c r="B21" s="33"/>
-      <c r="D21" s="37"/>
+      <c r="B21" s="29"/>
+      <c r="D21" s="33"/>
       <c r="E21" s="18"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="37"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="33"/>
       <c r="I21" s="21"/>
       <c r="K21" s="18"/>
-      <c r="L21" s="37"/>
-      <c r="M21" s="37"/>
-      <c r="N21" s="37"/>
-      <c r="O21" s="37"/>
-      <c r="P21" s="37"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
+      <c r="P21" s="33"/>
       <c r="Q21" s="21"/>
-      <c r="V21" s="98"/>
+      <c r="V21" s="87"/>
     </row>
     <row r="22" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="31"/>
+      <c r="B22" s="27"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="30"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="14"/>
       <c r="I22" s="1"/>
       <c r="J22"/>
-      <c r="K22" s="32"/>
+      <c r="K22" s="28"/>
       <c r="M22"/>
       <c r="N22" s="1"/>
       <c r="O22" s="12"/>
       <c r="T22"/>
       <c r="U22"/>
-      <c r="V22" s="97"/>
+      <c r="V22" s="86"/>
       <c r="W22"/>
       <c r="X22"/>
     </row>
     <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="34" t="s">
         <v>89</v>
       </c>
       <c r="D23" s="17"/>
-      <c r="E23" s="35" t="s">
+      <c r="E23" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="F23" s="41" t="s">
+      <c r="F23" s="34" t="s">
         <v>93</v>
       </c>
       <c r="G23" s="17"/>
@@ -2545,34 +2569,34 @@
       <c r="L23" s="17"/>
       <c r="M23" s="17"/>
       <c r="N23" s="17"/>
-      <c r="O23" s="102"/>
-      <c r="P23" s="102"/>
-      <c r="Q23" s="102"/>
-      <c r="R23" s="102"/>
-      <c r="S23" s="103"/>
-      <c r="T23" s="103"/>
-      <c r="U23" s="103"/>
-      <c r="V23" s="104"/>
+      <c r="O23" s="91"/>
+      <c r="P23" s="91"/>
+      <c r="Q23" s="91"/>
+      <c r="R23" s="91"/>
+      <c r="S23" s="92"/>
+      <c r="T23" s="92"/>
+      <c r="U23" s="92"/>
+      <c r="V23" s="93"/>
       <c r="W23"/>
       <c r="X23"/>
     </row>
     <row r="24" spans="1:24" s="20" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="B24" s="21"/>
-      <c r="D24" s="37"/>
+      <c r="D24" s="33"/>
       <c r="F24" s="15"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
       <c r="L24" s="21"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="37"/>
-      <c r="O24" s="37"/>
-      <c r="P24" s="37"/>
+      <c r="M24" s="33"/>
+      <c r="N24" s="33"/>
+      <c r="O24" s="33"/>
+      <c r="P24" s="33"/>
       <c r="R24" s="21"/>
       <c r="S24" s="21"/>
-      <c r="V24" s="98"/>
+      <c r="V24" s="87"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="E25" s="1"/>
@@ -2930,7 +2954,7 @@
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations disablePrompts="1" count="4">
     <dataValidation showErrorMessage="1" sqref="K4 F23 C20 C17 S17 L17 F17 F20 C23 L20 S20" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="G16 H11:H13" xr:uid="{00000000-0002-0000-0000-000002000000}">

</xml_diff>

<commit_message>
updated protocol sheets for reserves
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/Protocol-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5608072-C9DF-40CE-AEE1-967763E8FBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA09E098-E0F4-40D4-A193-2FE1A0318579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="9690" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5625" yWindow="4665" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="97">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -421,16 +421,22 @@
     <t>${session.announcerAsTO} ${session.announcerAsTO.federationId}</t>
   </si>
   <si>
+    <t>${session.reserveAsTO} ${session.reserveAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${group.item.category}</t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.reserveJuryAsTO} ${session.reserveJuryAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("ReserveJury")}</t>
+  </si>
+  <si>
     <t>${t.get("Reserve")}</t>
-  </si>
-  <si>
-    <t>${session.reserveAsTO} ${session.reserveAsTO.federationId}</t>
-  </si>
-  <si>
-    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId} ${session.reserveJuryAsTO != null ? "("+t.get("Reserve")+") "+session.reserveJuryAsTO+" "+session.reserveJuryAsTO.federationId : ""}</t>
-  </si>
-  <si>
-    <t>${group.item.category}</t>
   </si>
 </sst>
 </file>
@@ -1041,7 +1047,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1111,20 +1117,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1260,7 +1257,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1275,14 +1271,63 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1324,72 +1369,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1897,99 +1893,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
       <c r="G1" s="15"/>
-      <c r="J1" s="28" t="s">
+      <c r="J1" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="K1" s="94" t="s">
+      <c r="K1" s="105" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="94"/>
-      <c r="M1" s="94"/>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="94"/>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="94"/>
-      <c r="V1" s="94"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
+      <c r="P1" s="105"/>
+      <c r="Q1" s="105"/>
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="105"/>
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="46"/>
+      <c r="B2" s="43"/>
       <c r="C2" s="4"/>
-      <c r="J2" s="28" t="s">
+      <c r="J2" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="47" t="s">
+      <c r="K2" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="88"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="50"/>
-      <c r="R2" s="28" t="s">
+      <c r="L2" s="84"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="26" t="s">
         <v>30</v>
       </c>
       <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="50"/>
-      <c r="U2" s="50"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
     </row>
     <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="J3" s="28" t="s">
+      <c r="B3" s="49"/>
+      <c r="J3" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="108" t="s">
+      <c r="K3" s="122" t="s">
         <v>56</v>
       </c>
-      <c r="L3" s="108"/>
-      <c r="M3" s="108"/>
-      <c r="N3" s="108"/>
-      <c r="O3" s="108"/>
+      <c r="L3" s="122"/>
+      <c r="M3" s="122"/>
+      <c r="N3" s="122"/>
+      <c r="O3" s="122"/>
       <c r="P3" s="6"/>
-      <c r="Q3" s="53"/>
-      <c r="R3" s="28" t="s">
+      <c r="Q3" s="50"/>
+      <c r="R3" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="S3" s="54" t="s">
+      <c r="S3" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="T3" s="55"/>
-      <c r="U3" s="55"/>
-      <c r="V3" s="85"/>
+      <c r="T3" s="52"/>
+      <c r="U3" s="52"/>
+      <c r="V3" s="82"/>
     </row>
     <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="40"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="37"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
-      <c r="J4" s="28" t="s">
+      <c r="J4" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="89" t="s">
+      <c r="K4" s="85" t="s">
         <v>80</v>
       </c>
       <c r="L4"/>
@@ -1997,8 +1993,8 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="Q4"/>
-      <c r="R4" s="28"/>
-      <c r="S4" s="56"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="53"/>
     </row>
     <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2007,32 +2003,32 @@
       <c r="H6" s="7"/>
       <c r="I6" s="9"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="101" t="s">
+      <c r="K6" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="102"/>
-      <c r="M6" s="103"/>
-      <c r="N6" s="35" t="s">
+      <c r="L6" s="112"/>
+      <c r="M6" s="113"/>
+      <c r="N6" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="O6" s="101" t="s">
+      <c r="O6" s="111" t="s">
         <v>39</v>
       </c>
-      <c r="P6" s="102"/>
-      <c r="Q6" s="103"/>
-      <c r="R6" s="37" t="s">
+      <c r="P6" s="112"/>
+      <c r="Q6" s="113"/>
+      <c r="R6" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="S6" s="98" t="s">
+      <c r="S6" s="108" t="s">
         <v>45</v>
       </c>
-      <c r="T6" s="96" t="s">
+      <c r="T6" s="106" t="s">
         <v>46</v>
       </c>
-      <c r="U6" s="104" t="s">
+      <c r="U6" s="114" t="s">
         <v>81</v>
       </c>
-      <c r="V6" s="105"/>
+      <c r="V6" s="115"/>
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2048,10 +2044,10 @@
       <c r="D7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="101" t="s">
+      <c r="E7" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="103"/>
+      <c r="F7" s="113"/>
       <c r="G7" s="11" t="s">
         <v>34</v>
       </c>
@@ -2073,7 +2069,7 @@
       <c r="M7" s="10">
         <v>3</v>
       </c>
-      <c r="N7" s="36" t="s">
+      <c r="N7" s="33" t="s">
         <v>44</v>
       </c>
       <c r="O7" s="10">
@@ -2085,309 +2081,282 @@
       <c r="Q7" s="10">
         <v>3</v>
       </c>
-      <c r="R7" s="38" t="s">
+      <c r="R7" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="S7" s="99"/>
-      <c r="T7" s="97"/>
-      <c r="U7" s="106"/>
-      <c r="V7" s="107"/>
+      <c r="S7" s="109"/>
+      <c r="T7" s="107"/>
+      <c r="U7" s="116"/>
+      <c r="V7" s="117"/>
     </row>
     <row r="8" spans="1:24" s="25" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="57"/>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
-      <c r="I8" s="57"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="59"/>
+      <c r="A8" s="54"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="56"/>
     </row>
     <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="60" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="61"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
-      <c r="F9" s="62"/>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="62"/>
-      <c r="J9" s="62"/>
-      <c r="K9" s="62"/>
-      <c r="L9" s="62"/>
-      <c r="M9" s="62"/>
-      <c r="N9" s="62"/>
-      <c r="O9" s="62"/>
-      <c r="P9" s="62"/>
-      <c r="Q9" s="62"/>
-      <c r="R9" s="62"/>
-      <c r="S9" s="62"/>
-      <c r="T9" s="62"/>
-      <c r="U9" s="62"/>
-      <c r="V9" s="90"/>
+      <c r="A9" s="57" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="58"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="59"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="59"/>
+      <c r="P9" s="59"/>
+      <c r="Q9" s="59"/>
+      <c r="R9" s="59"/>
+      <c r="S9" s="59"/>
+      <c r="T9" s="59"/>
+      <c r="U9" s="59"/>
+      <c r="V9" s="86"/>
       <c r="X9"/>
     </row>
     <row r="10" spans="1:24" s="25" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="117" t="s">
+      <c r="A10" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="117" t="s">
+      <c r="B10" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="117" t="s">
+      <c r="C10" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="111" t="s">
+      <c r="D10" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="112" t="s">
+      <c r="E10" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="113"/>
-      <c r="G10" s="118" t="s">
+      <c r="F10" s="121"/>
+      <c r="G10" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="119" t="s">
+      <c r="H10" s="92" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="120" t="s">
+      <c r="I10" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="121" t="s">
+      <c r="J10" s="94" t="s">
         <v>26</v>
       </c>
-      <c r="K10" s="122" t="s">
+      <c r="K10" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="L10" s="122" t="s">
+      <c r="L10" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="M10" s="122" t="s">
+      <c r="M10" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="N10" s="123" t="s">
+      <c r="N10" s="96" t="s">
         <v>8</v>
       </c>
-      <c r="O10" s="122" t="s">
+      <c r="O10" s="95" t="s">
         <v>13</v>
       </c>
-      <c r="P10" s="122" t="s">
+      <c r="P10" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="Q10" s="122" t="s">
+      <c r="Q10" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="124" t="s">
+      <c r="R10" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="S10" s="125" t="s">
+      <c r="S10" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="T10" s="126" t="s">
+      <c r="T10" s="99" t="s">
         <v>78</v>
       </c>
-      <c r="U10" s="127" t="s">
+      <c r="U10" s="118" t="s">
         <v>82</v>
       </c>
-      <c r="V10" s="128"/>
+      <c r="V10" s="119"/>
     </row>
     <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="114"/>
-      <c r="C11" s="114"/>
-      <c r="D11" s="114"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="114"/>
-      <c r="G11" s="114"/>
-      <c r="H11" s="114"/>
-      <c r="I11" s="114"/>
-      <c r="J11" s="115"/>
-      <c r="K11" s="114"/>
-      <c r="L11" s="114"/>
-      <c r="M11" s="114"/>
-      <c r="N11" s="114"/>
-      <c r="O11" s="114"/>
-      <c r="P11" s="114"/>
-      <c r="Q11" s="114"/>
-      <c r="R11" s="114"/>
-      <c r="S11" s="114"/>
-      <c r="T11" s="114"/>
-      <c r="U11" s="114"/>
-      <c r="V11" s="114"/>
+      <c r="B11"/>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="O11"/>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
       <c r="W11"/>
       <c r="X11"/>
     </row>
-    <row r="12" spans="1:24" s="41" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
+    <row r="12" spans="1:24" s="38" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="110"/>
-      <c r="C12" s="110"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="110"/>
-      <c r="F12" s="110"/>
-      <c r="G12" s="110"/>
-      <c r="H12" s="110"/>
-      <c r="I12" s="110"/>
-      <c r="J12" s="116"/>
-      <c r="K12" s="110"/>
-      <c r="L12" s="110"/>
-      <c r="M12" s="110"/>
-      <c r="N12" s="110"/>
-      <c r="O12" s="110"/>
-      <c r="P12" s="110"/>
-      <c r="Q12" s="110"/>
-      <c r="R12" s="110"/>
-      <c r="S12" s="110"/>
-      <c r="T12" s="110"/>
-      <c r="U12" s="110"/>
-      <c r="V12" s="110"/>
-    </row>
-    <row r="13" spans="1:24" s="41" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="64"/>
-      <c r="B13" s="64"/>
-      <c r="C13" s="64"/>
-      <c r="D13" s="64"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="64"/>
-      <c r="G13" s="64"/>
-      <c r="H13" s="64"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="70"/>
-      <c r="K13" s="64"/>
-      <c r="L13" s="64"/>
-      <c r="M13" s="64"/>
-      <c r="N13" s="64"/>
-      <c r="O13" s="64"/>
-      <c r="P13" s="70"/>
-      <c r="Q13" s="70"/>
-      <c r="R13" s="70"/>
-      <c r="S13" s="64"/>
-      <c r="T13" s="64"/>
-      <c r="U13" s="70"/>
-      <c r="V13" s="70"/>
-    </row>
-    <row r="14" spans="1:24" s="82" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A14" s="73" t="s">
+      <c r="J12" s="39"/>
+    </row>
+    <row r="13" spans="1:24" s="38" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="61"/>
+      <c r="B13" s="61"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="61"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="61"/>
+      <c r="J13" s="67"/>
+      <c r="K13" s="61"/>
+      <c r="L13" s="61"/>
+      <c r="M13" s="61"/>
+      <c r="N13" s="61"/>
+      <c r="O13" s="61"/>
+      <c r="P13" s="67"/>
+      <c r="Q13" s="67"/>
+      <c r="R13" s="67"/>
+      <c r="S13" s="61"/>
+      <c r="T13" s="61"/>
+      <c r="U13" s="67"/>
+      <c r="V13" s="67"/>
+    </row>
+    <row r="14" spans="1:24" s="79" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A14" s="70" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="74"/>
-      <c r="C14" s="75"/>
-      <c r="D14" s="76" t="s">
+      <c r="B14" s="71"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="77" t="s">
+      <c r="E14" s="74" t="s">
         <v>71</v>
       </c>
-      <c r="F14" s="76" t="s">
+      <c r="F14" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="G14" s="78" t="s">
+      <c r="G14" s="75" t="s">
         <v>73</v>
       </c>
-      <c r="H14" s="79"/>
-      <c r="I14" s="76" t="s">
+      <c r="H14" s="76"/>
+      <c r="I14" s="73" t="s">
         <v>68</v>
       </c>
-      <c r="J14" s="73" t="s">
+      <c r="J14" s="70" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="80"/>
-      <c r="L14" s="74"/>
-      <c r="M14" s="75"/>
-      <c r="N14" s="73" t="s">
+      <c r="K14" s="77"/>
+      <c r="L14" s="71"/>
+      <c r="M14" s="72"/>
+      <c r="N14" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="O14" s="74"/>
-      <c r="P14" s="81"/>
-      <c r="Q14" s="73" t="s">
+      <c r="O14" s="71"/>
+      <c r="P14" s="78"/>
+      <c r="Q14" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="74"/>
-      <c r="S14" s="73" t="s">
+      <c r="R14" s="71"/>
+      <c r="S14" s="70" t="s">
         <v>65</v>
       </c>
-      <c r="T14" s="80"/>
-      <c r="U14" s="73" t="s">
+      <c r="T14" s="77"/>
+      <c r="U14" s="70" t="s">
         <v>69</v>
       </c>
-      <c r="V14" s="81"/>
-      <c r="X14" s="75"/>
-    </row>
-    <row r="15" spans="1:24" s="63" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="65" t="s">
+      <c r="V14" s="78"/>
+      <c r="X14" s="72"/>
+    </row>
+    <row r="15" spans="1:24" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="66"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="68" t="s">
+      <c r="B15" s="63"/>
+      <c r="C15" s="64"/>
+      <c r="D15" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="69" t="s">
+      <c r="E15" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="84" t="s">
+      <c r="F15" s="81" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="69" t="s">
+      <c r="G15" s="66" t="s">
         <v>77</v>
       </c>
-      <c r="H15" s="67"/>
-      <c r="I15" s="83" t="s">
+      <c r="H15" s="64"/>
+      <c r="I15" s="80" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="69" t="s">
+      <c r="J15" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="K15" s="66"/>
-      <c r="L15" s="66"/>
-      <c r="M15" s="67"/>
-      <c r="N15" s="69" t="s">
+      <c r="K15" s="63"/>
+      <c r="L15" s="63"/>
+      <c r="M15" s="64"/>
+      <c r="N15" s="66" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="66"/>
-      <c r="P15" s="67"/>
-      <c r="Q15" s="65" t="s">
+      <c r="O15" s="63"/>
+      <c r="P15" s="64"/>
+      <c r="Q15" s="62" t="s">
         <v>63</v>
       </c>
-      <c r="R15" s="66"/>
-      <c r="S15" s="72" t="s">
+      <c r="R15" s="63"/>
+      <c r="S15" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="T15" s="66"/>
-      <c r="U15" s="71" t="s">
+      <c r="T15" s="63"/>
+      <c r="U15" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="V15" s="67"/>
-      <c r="X15" s="67"/>
+      <c r="V15" s="64"/>
+      <c r="X15" s="64"/>
     </row>
     <row r="16" spans="1:24" s="13" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="109" t="s">
+      <c r="E16" s="104" t="s">
         <v>48</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="15"/>
       <c r="I16" s="14"/>
-      <c r="J16" s="95" t="s">
+      <c r="J16" s="103" t="s">
         <v>49</v>
       </c>
-      <c r="K16" s="95"/>
+      <c r="K16" s="103"/>
       <c r="L16" s="14"/>
       <c r="N16" s="16"/>
       <c r="P16" s="14"/>
-      <c r="Q16" s="100" t="s">
+      <c r="Q16" s="110" t="s">
         <v>50</v>
       </c>
-      <c r="R16" s="100"/>
-      <c r="S16" s="39"/>
+      <c r="R16" s="110"/>
+      <c r="S16" s="36"/>
       <c r="T16" s="14"/>
       <c r="U16" s="12"/>
       <c r="V16" s="16"/>
@@ -2398,77 +2367,77 @@
     </row>
     <row r="17" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="31" t="s">
         <v>90</v>
       </c>
       <c r="D17" s="17"/>
-      <c r="E17" s="109"/>
-      <c r="F17" s="34" t="s">
+      <c r="E17" s="104"/>
+      <c r="F17" s="31" t="s">
         <v>86</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
-      <c r="J17" s="95"/>
-      <c r="K17" s="95"/>
-      <c r="L17" s="34" t="s">
+      <c r="J17" s="103"/>
+      <c r="K17" s="103"/>
+      <c r="L17" s="31" t="s">
         <v>87</v>
       </c>
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
       <c r="O17" s="17"/>
       <c r="P17" s="19"/>
-      <c r="Q17" s="100"/>
-      <c r="R17" s="100"/>
-      <c r="S17" s="34" t="s">
+      <c r="Q17" s="110"/>
+      <c r="R17" s="110"/>
+      <c r="S17" s="31" t="s">
         <v>88</v>
       </c>
       <c r="T17" s="19"/>
       <c r="U17" s="17"/>
-      <c r="V17" s="43"/>
+      <c r="V17" s="40"/>
       <c r="W17"/>
     </row>
     <row r="18" spans="1:24" s="20" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="A18" s="21"/>
-      <c r="B18" s="29"/>
-      <c r="D18" s="33"/>
+      <c r="B18" s="27"/>
+      <c r="D18" s="30"/>
       <c r="E18" s="18"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="30"/>
       <c r="I18" s="21"/>
       <c r="K18" s="18"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
-      <c r="N18" s="33"/>
-      <c r="O18" s="33"/>
-      <c r="P18" s="33"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="30"/>
+      <c r="P18" s="30"/>
       <c r="Q18" s="21"/>
-      <c r="S18" s="33"/>
-      <c r="T18" s="33"/>
-      <c r="U18" s="33"/>
-      <c r="V18" s="87"/>
+      <c r="S18" s="30"/>
+      <c r="T18" s="30"/>
+      <c r="U18" s="30"/>
+      <c r="V18" s="83"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="27"/>
+      <c r="B19" s="100"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="26"/>
+      <c r="E19" s="101"/>
       <c r="F19" s="14"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="95" t="s">
+      <c r="J19" s="103" t="s">
         <v>53</v>
       </c>
-      <c r="K19" s="95"/>
+      <c r="K19" s="103"/>
       <c r="M19"/>
       <c r="N19" s="1"/>
       <c r="O19" s="12"/>
-      <c r="Q19" s="95" t="s">
-        <v>91</v>
-      </c>
-      <c r="R19" s="95"/>
+      <c r="Q19" s="103" t="s">
+        <v>96</v>
+      </c>
+      <c r="R19" s="103"/>
       <c r="S19" s="1"/>
       <c r="T19"/>
       <c r="V19" s="12"/>
@@ -2476,127 +2445,120 @@
     </row>
     <row r="20" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="17"/>
-      <c r="E20" s="31" t="s">
+      <c r="D20" s="87"/>
+      <c r="E20" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="F20" s="34" t="s">
+      <c r="F20" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="95"/>
-      <c r="K20" s="95"/>
-      <c r="L20" s="34" t="s">
+      <c r="G20" s="87"/>
+      <c r="H20" s="87"/>
+      <c r="I20" s="87"/>
+      <c r="J20" s="103"/>
+      <c r="K20" s="103"/>
+      <c r="L20" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="M20" s="19"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="95"/>
-      <c r="R20" s="95"/>
-      <c r="S20" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="T20" s="19"/>
-      <c r="U20" s="17"/>
-      <c r="V20" s="17"/>
+      <c r="M20" s="88"/>
+      <c r="N20" s="87"/>
+      <c r="O20" s="87"/>
+      <c r="P20" s="87"/>
+      <c r="Q20" s="103"/>
+      <c r="R20" s="103"/>
+      <c r="S20" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="T20" s="88"/>
+      <c r="U20" s="87"/>
+      <c r="V20" s="87"/>
       <c r="X20"/>
     </row>
     <row r="21" spans="1:24" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
-      <c r="B21" s="29"/>
-      <c r="D21" s="33"/>
+      <c r="B21" s="27"/>
       <c r="E21" s="18"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="33"/>
+      <c r="F21" s="102"/>
       <c r="I21" s="21"/>
       <c r="K21" s="18"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
-      <c r="N21" s="33"/>
-      <c r="O21" s="33"/>
-      <c r="P21" s="33"/>
       <c r="Q21" s="21"/>
-      <c r="V21" s="87"/>
+      <c r="V21" s="83"/>
     </row>
     <row r="22" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="27"/>
+      <c r="A22" s="104" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" s="104"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="26"/>
+      <c r="E22" s="101"/>
       <c r="F22" s="14"/>
       <c r="I22" s="1"/>
       <c r="J22"/>
-      <c r="K22" s="28"/>
+      <c r="K22" s="26"/>
       <c r="M22"/>
       <c r="N22" s="1"/>
       <c r="O22" s="12"/>
+      <c r="Q22" s="104" t="s">
+        <v>95</v>
+      </c>
+      <c r="R22" s="104"/>
+      <c r="S22" s="1"/>
       <c r="T22"/>
-      <c r="U22"/>
-      <c r="V22" s="86"/>
+      <c r="V22" s="12"/>
       <c r="W22"/>
       <c r="X22"/>
     </row>
     <row r="23" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C23" s="34" t="s">
+      <c r="A23" s="104"/>
+      <c r="B23" s="104"/>
+      <c r="C23" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="17"/>
-      <c r="E23" s="31" t="s">
+      <c r="D23" s="87"/>
+      <c r="E23" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="F23" s="34" t="s">
+      <c r="F23" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="91"/>
-      <c r="P23" s="91"/>
-      <c r="Q23" s="91"/>
-      <c r="R23" s="91"/>
-      <c r="S23" s="92"/>
-      <c r="T23" s="92"/>
-      <c r="U23" s="92"/>
-      <c r="V23" s="93"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="87"/>
+      <c r="I23" s="87"/>
+      <c r="J23" s="87"/>
+      <c r="K23" s="87"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="87"/>
+      <c r="N23" s="87"/>
+      <c r="O23" s="87"/>
+      <c r="Q23" s="104"/>
+      <c r="R23" s="104"/>
+      <c r="S23" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="T23" s="88"/>
+      <c r="U23" s="87"/>
+      <c r="V23" s="87"/>
       <c r="W23"/>
       <c r="X23"/>
     </row>
     <row r="24" spans="1:24" s="20" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="B24" s="21"/>
-      <c r="D24" s="33"/>
       <c r="F24" s="15"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30"/>
+      <c r="G24" s="102"/>
+      <c r="H24" s="102"/>
+      <c r="I24" s="102"/>
+      <c r="J24" s="102"/>
+      <c r="K24" s="102"/>
       <c r="L24" s="21"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
       <c r="R24" s="21"/>
       <c r="S24" s="21"/>
-      <c r="V24" s="87"/>
+      <c r="V24" s="83"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="E25" s="1"/>
@@ -2922,12 +2884,10 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="15">
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="K3:O3"/>
+  <mergeCells count="17">
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="J16:K17"/>
+    <mergeCell ref="A22:B23"/>
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="J19:K20"/>
     <mergeCell ref="T6:T7"/>
@@ -2938,6 +2898,10 @@
     <mergeCell ref="U6:V7"/>
     <mergeCell ref="U10:V10"/>
     <mergeCell ref="Q19:R20"/>
+    <mergeCell ref="Q22:R23"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="K3:O3"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:D8">
     <cfRule type="expression" dxfId="2" priority="7" stopIfTrue="1">
@@ -2954,8 +2918,8 @@
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="4">
-    <dataValidation showErrorMessage="1" sqref="K4 F23 C20 C17 S17 L17 F17 F20 C23 L20 S20" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+  <dataValidations count="4">
+    <dataValidation showErrorMessage="1" sqref="K4 F23 C20 C17 S17 L17 F17 F20 C23 L20 S20 S23" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="G16 H11:H13" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>

</xml_diff>